<commit_message>
feat: add 'uom' field to MtcKebutuhanMaterial
- Updated MtcSipilController to include 'uom' in the store method.
- Enhanced MtcKebutuhanMaterialRequest to validate 'uom' for materials.
- Modified MtcKebutuhanMaterialModel to include 'uom' in fillable attributes.
- Altered migration to add 'uom' column to mtc_kebutuhan_material table.
- Updated various Excel templates in the maintenance directory.
</commit_message>
<xml_diff>
--- a/public/assets/templates/maintenance/electric_engine.xlsx
+++ b/public/assets/templates/maintenance/electric_engine.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\laragon\www\pt_bas\Engineering\public\assets\templates\maintenance\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F4C6ADB1-3B10-40FC-9AB3-0B29888F5D20}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8FC6B1D4-6BBE-4CD9-A85F-D187281B8196}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10560" xr2:uid="{7A80608D-5162-4C69-AACA-06EF8CFA5F02}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="ELECTRIC ENGINE" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'ELECTRIC ENGINE'!$A$1:$I$75</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'ELECTRIC ENGINE'!$A$1:$I$78</definedName>
   </definedNames>
   <calcPr calcId="191029" concurrentCalc="0"/>
   <extLst>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="117" uniqueCount="74">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="127" uniqueCount="79">
   <si>
     <t>LAPORAN MAINTENANCE ELECTRIC ENGINE</t>
   </si>
@@ -42,15 +42,9 @@
     <t>Nama Mesin</t>
   </si>
   <si>
-    <t xml:space="preserve">Waktu   </t>
-  </si>
-  <si>
     <t>Running Hour</t>
   </si>
   <si>
-    <t xml:space="preserve">:  </t>
-  </si>
-  <si>
     <t>Mesin</t>
   </si>
   <si>
@@ -250,6 +244,27 @@
   </si>
   <si>
     <t xml:space="preserve">Tanggal </t>
+  </si>
+  <si>
+    <t>Waktu Mulai</t>
+  </si>
+  <si>
+    <t>Waktu Selesai</t>
+  </si>
+  <si>
+    <t xml:space="preserve">: </t>
+  </si>
+  <si>
+    <t>Kode Mesin</t>
+  </si>
+  <si>
+    <t>Lokasi</t>
+  </si>
+  <si>
+    <t>Paket</t>
+  </si>
+  <si>
+    <t>Departemen</t>
   </si>
 </sst>
 </file>
@@ -657,7 +672,7 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="79">
+  <cellXfs count="84">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -736,6 +751,21 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -793,9 +823,6 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -820,6 +847,33 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
@@ -868,32 +922,8 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1262,7 +1292,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BC5D322C-4578-4471-B9FD-0A0DA5343548}">
-  <dimension ref="A1:M83"/>
+  <dimension ref="A1:M86"/>
   <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="11" style="21" customWidth="1"/>
@@ -1277,1105 +1307,1125 @@
     <col min="13" max="13" width="10.7265625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" ht="15" thickTop="1">
-      <c r="A1" s="29"/>
-      <c r="B1" s="30"/>
-      <c r="C1" s="30"/>
-      <c r="D1" s="33" t="s">
+    <row r="1" spans="1:9" ht="15" thickTop="1">
+      <c r="A1" s="34"/>
+      <c r="B1" s="35"/>
+      <c r="C1" s="35"/>
+      <c r="D1" s="38" t="s">
         <v>0</v>
       </c>
-      <c r="E1" s="33"/>
-      <c r="F1" s="33"/>
-      <c r="G1" s="33"/>
-      <c r="H1" s="33"/>
-      <c r="I1" s="34"/>
-    </row>
-    <row r="2" spans="1:13">
-      <c r="A2" s="31"/>
-      <c r="B2" s="32"/>
-      <c r="C2" s="32"/>
-      <c r="D2" s="35" t="s">
+      <c r="E1" s="38"/>
+      <c r="F1" s="38"/>
+      <c r="G1" s="38"/>
+      <c r="H1" s="38"/>
+      <c r="I1" s="39"/>
+    </row>
+    <row r="2" spans="1:9">
+      <c r="A2" s="36"/>
+      <c r="B2" s="37"/>
+      <c r="C2" s="37"/>
+      <c r="D2" s="40" t="s">
         <v>1</v>
       </c>
-      <c r="E2" s="35"/>
-      <c r="F2" s="35"/>
-      <c r="G2" s="35"/>
-      <c r="H2" s="35"/>
-      <c r="I2" s="36"/>
-    </row>
-    <row r="3" spans="1:13" ht="10" customHeight="1">
+      <c r="E2" s="40"/>
+      <c r="F2" s="40"/>
+      <c r="G2" s="40"/>
+      <c r="H2" s="40"/>
+      <c r="I2" s="41"/>
+    </row>
+    <row r="3" spans="1:9" ht="10" customHeight="1">
       <c r="A3" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="B3" s="27" t="s">
+        <v>2</v>
+      </c>
+      <c r="C3" s="28"/>
+      <c r="D3" s="28"/>
+      <c r="E3" s="42" t="s">
+        <v>3</v>
+      </c>
+      <c r="F3" s="43"/>
+      <c r="G3" s="29" t="s">
+        <v>2</v>
+      </c>
+      <c r="H3" s="29"/>
+      <c r="I3" s="30"/>
+    </row>
+    <row r="4" spans="1:9" ht="10" customHeight="1">
+      <c r="A4" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="B4" s="27" t="s">
+        <v>74</v>
+      </c>
+      <c r="C4" s="28"/>
+      <c r="D4" s="28"/>
+      <c r="E4" s="28" t="s">
+        <v>75</v>
+      </c>
+      <c r="F4" s="28"/>
+      <c r="G4" s="29" t="s">
+        <v>74</v>
+      </c>
+      <c r="H4" s="29"/>
+      <c r="I4" s="30"/>
+    </row>
+    <row r="5" spans="1:9" ht="10" customHeight="1">
+      <c r="A5" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="B3" s="45" t="s">
+      <c r="B5" s="27" t="s">
+        <v>74</v>
+      </c>
+      <c r="C5" s="28"/>
+      <c r="D5" s="28"/>
+      <c r="E5" s="28" t="s">
+        <v>76</v>
+      </c>
+      <c r="F5" s="28"/>
+      <c r="G5" s="29" t="s">
+        <v>74</v>
+      </c>
+      <c r="H5" s="29"/>
+      <c r="I5" s="30"/>
+    </row>
+    <row r="6" spans="1:9" ht="10" customHeight="1">
+      <c r="A6" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="B6" s="26" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="45"/>
-      <c r="D3" s="45"/>
-      <c r="E3" s="37" t="s">
-        <v>3</v>
-      </c>
-      <c r="F3" s="38"/>
-      <c r="G3" s="39" t="s">
+      <c r="C6" s="28"/>
+      <c r="D6" s="28"/>
+      <c r="E6" s="42" t="s">
+        <v>4</v>
+      </c>
+      <c r="F6" s="43"/>
+      <c r="G6" s="29" t="s">
+        <v>74</v>
+      </c>
+      <c r="H6" s="29"/>
+      <c r="I6" s="30"/>
+    </row>
+    <row r="7" spans="1:9" ht="10" customHeight="1">
+      <c r="A7" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="B7" s="27" t="s">
         <v>2</v>
       </c>
-      <c r="H3" s="40"/>
-      <c r="I3" s="41"/>
-    </row>
-    <row r="4" spans="1:13" ht="10" customHeight="1">
-      <c r="A4" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="B4" s="45" t="s">
-        <v>2</v>
-      </c>
-      <c r="C4" s="45"/>
-      <c r="D4" s="45"/>
-      <c r="E4" s="37" t="s">
+      <c r="C7" s="28"/>
+      <c r="D7" s="28"/>
+      <c r="E7" s="83"/>
+      <c r="F7" s="83"/>
+      <c r="G7" s="44"/>
+      <c r="H7" s="45"/>
+      <c r="I7" s="46"/>
+    </row>
+    <row r="8" spans="1:9" s="5" customFormat="1" ht="11" customHeight="1">
+      <c r="A8" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="F4" s="38"/>
-      <c r="G4" s="39" t="s">
+      <c r="B8" s="47" t="s">
         <v>6</v>
       </c>
-      <c r="H4" s="40"/>
-      <c r="I4" s="41"/>
-    </row>
-    <row r="5" spans="1:13" s="5" customFormat="1" ht="11" customHeight="1">
-      <c r="A5" s="2" t="s">
+      <c r="C8" s="47"/>
+      <c r="D8" s="47"/>
+      <c r="E8" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="B5" s="42" t="s">
+      <c r="F8" s="48" t="s">
         <v>8</v>
       </c>
-      <c r="C5" s="42"/>
-      <c r="D5" s="42"/>
-      <c r="E5" s="3" t="s">
+      <c r="G8" s="48"/>
+      <c r="H8" s="48"/>
+      <c r="I8" s="49"/>
+    </row>
+    <row r="9" spans="1:9" s="9" customFormat="1" ht="9" customHeight="1">
+      <c r="A9" s="31" t="s">
         <v>9</v>
       </c>
-      <c r="F5" s="43" t="s">
-        <v>10</v>
-      </c>
-      <c r="G5" s="43"/>
-      <c r="H5" s="43"/>
-      <c r="I5" s="44"/>
-    </row>
-    <row r="6" spans="1:13" s="9" customFormat="1" ht="9" customHeight="1">
-      <c r="A6" s="26" t="s">
-        <v>11</v>
-      </c>
-      <c r="B6" s="6"/>
-      <c r="C6" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="D6" s="8" t="s">
-        <v>13</v>
-      </c>
-      <c r="E6" s="22"/>
-      <c r="F6" s="27"/>
-      <c r="G6" s="27"/>
-      <c r="H6" s="27"/>
-      <c r="I6" s="28"/>
-    </row>
-    <row r="7" spans="1:13" s="9" customFormat="1" ht="9" customHeight="1">
-      <c r="A7" s="26"/>
-      <c r="B7" s="6"/>
-      <c r="C7" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="D7" s="8" t="s">
-        <v>14</v>
-      </c>
-      <c r="E7" s="22"/>
-      <c r="F7" s="27"/>
-      <c r="G7" s="27"/>
-      <c r="H7" s="27"/>
-      <c r="I7" s="28"/>
-    </row>
-    <row r="8" spans="1:13" s="9" customFormat="1" ht="9" customHeight="1">
-      <c r="A8" s="26"/>
-      <c r="B8" s="6"/>
-      <c r="C8" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="D8" s="8" t="s">
-        <v>15</v>
-      </c>
-      <c r="E8" s="22"/>
-      <c r="F8" s="27"/>
-      <c r="G8" s="27"/>
-      <c r="H8" s="27"/>
-      <c r="I8" s="28"/>
-    </row>
-    <row r="9" spans="1:13" s="9" customFormat="1" ht="9" customHeight="1">
-      <c r="A9" s="26"/>
       <c r="B9" s="6"/>
       <c r="C9" s="7" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D9" s="8" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="E9" s="22"/>
-      <c r="F9" s="27"/>
-      <c r="G9" s="27"/>
-      <c r="H9" s="27"/>
-      <c r="I9" s="28"/>
-    </row>
-    <row r="10" spans="1:13" s="9" customFormat="1" ht="9" customHeight="1">
-      <c r="A10" s="26"/>
+      <c r="F9" s="32"/>
+      <c r="G9" s="32"/>
+      <c r="H9" s="32"/>
+      <c r="I9" s="33"/>
+    </row>
+    <row r="10" spans="1:9" s="9" customFormat="1" ht="9" customHeight="1">
+      <c r="A10" s="31"/>
       <c r="B10" s="6"/>
       <c r="C10" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="D10" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="D10" s="8" t="s">
-        <v>17</v>
-      </c>
       <c r="E10" s="22"/>
-      <c r="F10" s="27"/>
-      <c r="G10" s="27"/>
-      <c r="H10" s="27"/>
-      <c r="I10" s="28"/>
-    </row>
-    <row r="11" spans="1:13" s="9" customFormat="1" ht="9" customHeight="1">
-      <c r="A11" s="26"/>
+      <c r="F10" s="32"/>
+      <c r="G10" s="32"/>
+      <c r="H10" s="32"/>
+      <c r="I10" s="33"/>
+    </row>
+    <row r="11" spans="1:9" s="9" customFormat="1" ht="9" customHeight="1">
+      <c r="A11" s="31"/>
       <c r="B11" s="6"/>
       <c r="C11" s="7" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D11" s="8" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="E11" s="22"/>
-      <c r="F11" s="27"/>
-      <c r="G11" s="27"/>
-      <c r="H11" s="27"/>
-      <c r="I11" s="28"/>
-    </row>
-    <row r="12" spans="1:13" s="9" customFormat="1" ht="9" customHeight="1">
-      <c r="A12" s="26"/>
+      <c r="F11" s="32"/>
+      <c r="G11" s="32"/>
+      <c r="H11" s="32"/>
+      <c r="I11" s="33"/>
+    </row>
+    <row r="12" spans="1:9" s="9" customFormat="1" ht="9" customHeight="1">
+      <c r="A12" s="31"/>
       <c r="B12" s="6"/>
       <c r="C12" s="7" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D12" s="8" t="s">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="E12" s="22"/>
-      <c r="F12" s="27"/>
-      <c r="G12" s="27"/>
-      <c r="H12" s="27"/>
-      <c r="I12" s="28"/>
-    </row>
-    <row r="13" spans="1:13" s="9" customFormat="1" ht="9" customHeight="1">
-      <c r="A13" s="26"/>
+      <c r="F12" s="32"/>
+      <c r="G12" s="32"/>
+      <c r="H12" s="32"/>
+      <c r="I12" s="33"/>
+    </row>
+    <row r="13" spans="1:9" s="9" customFormat="1" ht="9" customHeight="1">
+      <c r="A13" s="31"/>
       <c r="B13" s="6"/>
       <c r="C13" s="7" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D13" s="8" t="s">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="E13" s="22"/>
-      <c r="F13" s="27"/>
-      <c r="G13" s="27"/>
-      <c r="H13" s="27"/>
-      <c r="I13" s="28"/>
-    </row>
-    <row r="14" spans="1:13" s="9" customFormat="1" ht="9" customHeight="1">
-      <c r="A14" s="26"/>
+      <c r="F13" s="32"/>
+      <c r="G13" s="32"/>
+      <c r="H13" s="32"/>
+      <c r="I13" s="33"/>
+    </row>
+    <row r="14" spans="1:9" s="9" customFormat="1" ht="9" customHeight="1">
+      <c r="A14" s="31"/>
       <c r="B14" s="6"/>
-      <c r="C14" s="7"/>
-      <c r="D14" s="8"/>
+      <c r="C14" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="D14" s="8" t="s">
+        <v>16</v>
+      </c>
       <c r="E14" s="22"/>
-      <c r="F14" s="27"/>
-      <c r="G14" s="27"/>
-      <c r="H14" s="27"/>
-      <c r="I14" s="28"/>
-    </row>
-    <row r="15" spans="1:13" s="9" customFormat="1" ht="9" customHeight="1">
-      <c r="A15" s="26"/>
+      <c r="F14" s="32"/>
+      <c r="G14" s="32"/>
+      <c r="H14" s="32"/>
+      <c r="I14" s="33"/>
+    </row>
+    <row r="15" spans="1:9" s="9" customFormat="1" ht="9" customHeight="1">
+      <c r="A15" s="31"/>
       <c r="B15" s="6"/>
+      <c r="C15" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="D15" s="8" t="s">
+        <v>17</v>
+      </c>
       <c r="E15" s="22"/>
-      <c r="F15" s="27"/>
-      <c r="G15" s="27"/>
-      <c r="H15" s="27"/>
-      <c r="I15" s="28"/>
-    </row>
-    <row r="16" spans="1:13" s="9" customFormat="1" ht="9" customHeight="1">
-      <c r="A16" s="47" t="s">
-        <v>21</v>
-      </c>
+      <c r="F15" s="32"/>
+      <c r="G15" s="32"/>
+      <c r="H15" s="32"/>
+      <c r="I15" s="33"/>
+    </row>
+    <row r="16" spans="1:9" s="9" customFormat="1" ht="9" customHeight="1">
+      <c r="A16" s="31"/>
       <c r="B16" s="6"/>
       <c r="C16" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="D16" s="10" t="s">
-        <v>22</v>
+        <v>10</v>
+      </c>
+      <c r="D16" s="8" t="s">
+        <v>18</v>
       </c>
       <c r="E16" s="22"/>
-      <c r="F16" s="27"/>
-      <c r="G16" s="27"/>
-      <c r="H16" s="27"/>
-      <c r="I16" s="28"/>
-      <c r="L16" s="48"/>
-      <c r="M16" s="48"/>
+      <c r="F16" s="32"/>
+      <c r="G16" s="32"/>
+      <c r="H16" s="32"/>
+      <c r="I16" s="33"/>
     </row>
     <row r="17" spans="1:13" s="9" customFormat="1" ht="9" customHeight="1">
-      <c r="A17" s="47"/>
+      <c r="A17" s="31"/>
       <c r="B17" s="6"/>
-      <c r="C17" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="D17" s="8" t="s">
-        <v>23</v>
-      </c>
+      <c r="C17" s="7"/>
+      <c r="D17" s="8"/>
       <c r="E17" s="22"/>
-      <c r="F17" s="27"/>
-      <c r="G17" s="27"/>
-      <c r="H17" s="27"/>
-      <c r="I17" s="28"/>
-      <c r="L17" s="49"/>
-      <c r="M17" s="49"/>
+      <c r="F17" s="32"/>
+      <c r="G17" s="32"/>
+      <c r="H17" s="32"/>
+      <c r="I17" s="33"/>
     </row>
     <row r="18" spans="1:13" s="9" customFormat="1" ht="9" customHeight="1">
-      <c r="A18" s="47"/>
+      <c r="A18" s="31"/>
       <c r="B18" s="6"/>
-      <c r="C18" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="D18" s="8" t="s">
-        <v>24</v>
-      </c>
       <c r="E18" s="22"/>
-      <c r="F18" s="27"/>
-      <c r="G18" s="27"/>
-      <c r="H18" s="27"/>
-      <c r="I18" s="28"/>
-      <c r="L18" s="49"/>
-      <c r="M18" s="49"/>
+      <c r="F18" s="32"/>
+      <c r="G18" s="32"/>
+      <c r="H18" s="32"/>
+      <c r="I18" s="33"/>
     </row>
     <row r="19" spans="1:13" s="9" customFormat="1" ht="9" customHeight="1">
-      <c r="A19" s="47"/>
+      <c r="A19" s="51" t="s">
+        <v>19</v>
+      </c>
       <c r="B19" s="6"/>
       <c r="C19" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="D19" s="8" t="s">
-        <v>25</v>
+        <v>10</v>
+      </c>
+      <c r="D19" s="10" t="s">
+        <v>20</v>
       </c>
       <c r="E19" s="22"/>
-      <c r="F19" s="27"/>
-      <c r="G19" s="27"/>
-      <c r="H19" s="27"/>
-      <c r="I19" s="28"/>
+      <c r="F19" s="32"/>
+      <c r="G19" s="32"/>
+      <c r="H19" s="32"/>
+      <c r="I19" s="33"/>
+      <c r="L19" s="52"/>
+      <c r="M19" s="52"/>
     </row>
     <row r="20" spans="1:13" s="9" customFormat="1" ht="9" customHeight="1">
-      <c r="A20" s="47"/>
+      <c r="A20" s="51"/>
       <c r="B20" s="6"/>
       <c r="C20" s="7" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D20" s="8" t="s">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="E20" s="22"/>
-      <c r="F20" s="27"/>
-      <c r="G20" s="27"/>
-      <c r="H20" s="27"/>
-      <c r="I20" s="28"/>
+      <c r="F20" s="32"/>
+      <c r="G20" s="32"/>
+      <c r="H20" s="32"/>
+      <c r="I20" s="33"/>
+      <c r="L20" s="53"/>
+      <c r="M20" s="53"/>
     </row>
     <row r="21" spans="1:13" s="9" customFormat="1" ht="9" customHeight="1">
-      <c r="A21" s="47"/>
+      <c r="A21" s="51"/>
       <c r="B21" s="6"/>
       <c r="C21" s="7" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D21" s="8" t="s">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="E21" s="22"/>
-      <c r="F21" s="27"/>
-      <c r="G21" s="27"/>
-      <c r="H21" s="27"/>
-      <c r="I21" s="28"/>
+      <c r="F21" s="32"/>
+      <c r="G21" s="32"/>
+      <c r="H21" s="32"/>
+      <c r="I21" s="33"/>
+      <c r="L21" s="53"/>
+      <c r="M21" s="53"/>
     </row>
     <row r="22" spans="1:13" s="9" customFormat="1" ht="9" customHeight="1">
-      <c r="A22" s="47"/>
+      <c r="A22" s="51"/>
       <c r="B22" s="6"/>
       <c r="C22" s="7" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D22" s="8" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="E22" s="22"/>
-      <c r="F22" s="27"/>
-      <c r="G22" s="27"/>
-      <c r="H22" s="27"/>
-      <c r="I22" s="28"/>
-      <c r="L22" s="46"/>
-      <c r="M22" s="46"/>
+      <c r="F22" s="32"/>
+      <c r="G22" s="32"/>
+      <c r="H22" s="32"/>
+      <c r="I22" s="33"/>
     </row>
     <row r="23" spans="1:13" s="9" customFormat="1" ht="9" customHeight="1">
-      <c r="A23" s="47"/>
+      <c r="A23" s="51"/>
       <c r="B23" s="6"/>
       <c r="C23" s="7" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D23" s="8" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
       <c r="E23" s="22"/>
-      <c r="F23" s="27"/>
-      <c r="G23" s="27"/>
-      <c r="H23" s="27"/>
-      <c r="I23" s="28"/>
-      <c r="L23" s="46"/>
-      <c r="M23" s="46"/>
+      <c r="F23" s="32"/>
+      <c r="G23" s="32"/>
+      <c r="H23" s="32"/>
+      <c r="I23" s="33"/>
     </row>
     <row r="24" spans="1:13" s="9" customFormat="1" ht="9" customHeight="1">
-      <c r="A24" s="47"/>
+      <c r="A24" s="51"/>
       <c r="B24" s="6"/>
       <c r="C24" s="7" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D24" s="8" t="s">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="E24" s="22"/>
-      <c r="F24" s="27"/>
-      <c r="G24" s="27"/>
-      <c r="H24" s="27"/>
-      <c r="I24" s="28"/>
+      <c r="F24" s="32"/>
+      <c r="G24" s="32"/>
+      <c r="H24" s="32"/>
+      <c r="I24" s="33"/>
     </row>
     <row r="25" spans="1:13" s="9" customFormat="1" ht="9" customHeight="1">
-      <c r="A25" s="47"/>
+      <c r="A25" s="51"/>
       <c r="B25" s="6"/>
       <c r="C25" s="7" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D25" s="8" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="E25" s="22"/>
-      <c r="F25" s="27"/>
-      <c r="G25" s="27"/>
-      <c r="H25" s="27"/>
-      <c r="I25" s="28"/>
+      <c r="F25" s="32"/>
+      <c r="G25" s="32"/>
+      <c r="H25" s="32"/>
+      <c r="I25" s="33"/>
+      <c r="L25" s="50"/>
+      <c r="M25" s="50"/>
     </row>
     <row r="26" spans="1:13" s="9" customFormat="1" ht="9" customHeight="1">
-      <c r="A26" s="47"/>
+      <c r="A26" s="51"/>
       <c r="B26" s="6"/>
       <c r="C26" s="7" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D26" s="8" t="s">
-        <v>32</v>
+        <v>27</v>
       </c>
       <c r="E26" s="22"/>
-      <c r="F26" s="27"/>
-      <c r="G26" s="27"/>
-      <c r="H26" s="27"/>
-      <c r="I26" s="28"/>
-      <c r="L26" s="46"/>
-      <c r="M26" s="46"/>
+      <c r="F26" s="32"/>
+      <c r="G26" s="32"/>
+      <c r="H26" s="32"/>
+      <c r="I26" s="33"/>
+      <c r="L26" s="50"/>
+      <c r="M26" s="50"/>
     </row>
     <row r="27" spans="1:13" s="9" customFormat="1" ht="9" customHeight="1">
-      <c r="A27" s="47"/>
+      <c r="A27" s="51"/>
       <c r="B27" s="6"/>
       <c r="C27" s="7" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D27" s="8" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="E27" s="22"/>
-      <c r="F27" s="27"/>
-      <c r="G27" s="27"/>
-      <c r="H27" s="27"/>
-      <c r="I27" s="28"/>
-      <c r="L27" s="11"/>
-      <c r="M27" s="11"/>
+      <c r="F27" s="32"/>
+      <c r="G27" s="32"/>
+      <c r="H27" s="32"/>
+      <c r="I27" s="33"/>
     </row>
     <row r="28" spans="1:13" s="9" customFormat="1" ht="9" customHeight="1">
-      <c r="A28" s="47"/>
+      <c r="A28" s="51"/>
       <c r="B28" s="6"/>
       <c r="C28" s="7" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D28" s="8" t="s">
-        <v>34</v>
+        <v>29</v>
       </c>
       <c r="E28" s="22"/>
-      <c r="F28" s="27"/>
-      <c r="G28" s="27"/>
-      <c r="H28" s="27"/>
-      <c r="I28" s="28"/>
-      <c r="L28" s="11"/>
-      <c r="M28" s="11"/>
+      <c r="F28" s="32"/>
+      <c r="G28" s="32"/>
+      <c r="H28" s="32"/>
+      <c r="I28" s="33"/>
     </row>
     <row r="29" spans="1:13" s="9" customFormat="1" ht="9" customHeight="1">
-      <c r="A29" s="47"/>
+      <c r="A29" s="51"/>
       <c r="B29" s="6"/>
+      <c r="C29" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="D29" s="8" t="s">
+        <v>30</v>
+      </c>
       <c r="E29" s="22"/>
-      <c r="F29" s="27"/>
-      <c r="G29" s="27"/>
-      <c r="H29" s="27"/>
-      <c r="I29" s="28"/>
+      <c r="F29" s="32"/>
+      <c r="G29" s="32"/>
+      <c r="H29" s="32"/>
+      <c r="I29" s="33"/>
+      <c r="L29" s="50"/>
+      <c r="M29" s="50"/>
     </row>
     <row r="30" spans="1:13" s="9" customFormat="1" ht="9" customHeight="1">
-      <c r="A30" s="47" t="s">
-        <v>35</v>
-      </c>
+      <c r="A30" s="51"/>
       <c r="B30" s="6"/>
       <c r="C30" s="7" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D30" s="8" t="s">
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="E30" s="22"/>
-      <c r="F30" s="27"/>
-      <c r="G30" s="27"/>
-      <c r="H30" s="27"/>
-      <c r="I30" s="28"/>
+      <c r="F30" s="32"/>
+      <c r="G30" s="32"/>
+      <c r="H30" s="32"/>
+      <c r="I30" s="33"/>
+      <c r="L30" s="11"/>
+      <c r="M30" s="11"/>
     </row>
     <row r="31" spans="1:13" s="9" customFormat="1" ht="9" customHeight="1">
-      <c r="A31" s="47"/>
+      <c r="A31" s="51"/>
       <c r="B31" s="6"/>
       <c r="C31" s="7" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D31" s="8" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="E31" s="22"/>
-      <c r="F31" s="27"/>
-      <c r="G31" s="27"/>
-      <c r="H31" s="27"/>
-      <c r="I31" s="28"/>
+      <c r="F31" s="32"/>
+      <c r="G31" s="32"/>
+      <c r="H31" s="32"/>
+      <c r="I31" s="33"/>
+      <c r="L31" s="11"/>
+      <c r="M31" s="11"/>
     </row>
     <row r="32" spans="1:13" s="9" customFormat="1" ht="9" customHeight="1">
-      <c r="A32" s="47"/>
+      <c r="A32" s="51"/>
       <c r="B32" s="6"/>
-      <c r="C32" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="D32" s="8" t="s">
-        <v>38</v>
-      </c>
       <c r="E32" s="22"/>
-      <c r="F32" s="27"/>
-      <c r="G32" s="27"/>
-      <c r="H32" s="27"/>
-      <c r="I32" s="28"/>
+      <c r="F32" s="32"/>
+      <c r="G32" s="32"/>
+      <c r="H32" s="32"/>
+      <c r="I32" s="33"/>
     </row>
     <row r="33" spans="1:9" s="9" customFormat="1" ht="9" customHeight="1">
-      <c r="A33" s="47"/>
+      <c r="A33" s="51" t="s">
+        <v>33</v>
+      </c>
       <c r="B33" s="6"/>
       <c r="C33" s="7" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D33" s="8" t="s">
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="E33" s="22"/>
-      <c r="F33" s="27"/>
-      <c r="G33" s="27"/>
-      <c r="H33" s="27"/>
-      <c r="I33" s="28"/>
+      <c r="F33" s="32"/>
+      <c r="G33" s="32"/>
+      <c r="H33" s="32"/>
+      <c r="I33" s="33"/>
     </row>
     <row r="34" spans="1:9" s="9" customFormat="1" ht="9" customHeight="1">
-      <c r="A34" s="47"/>
+      <c r="A34" s="51"/>
       <c r="B34" s="6"/>
       <c r="C34" s="7" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D34" s="8" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="E34" s="22"/>
-      <c r="F34" s="27"/>
-      <c r="G34" s="27"/>
-      <c r="H34" s="27"/>
-      <c r="I34" s="28"/>
+      <c r="F34" s="32"/>
+      <c r="G34" s="32"/>
+      <c r="H34" s="32"/>
+      <c r="I34" s="33"/>
     </row>
     <row r="35" spans="1:9" s="9" customFormat="1" ht="9" customHeight="1">
-      <c r="A35" s="47"/>
+      <c r="A35" s="51"/>
       <c r="B35" s="6"/>
       <c r="C35" s="7" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D35" s="8" t="s">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="E35" s="22"/>
-      <c r="F35" s="27"/>
-      <c r="G35" s="27"/>
-      <c r="H35" s="27"/>
-      <c r="I35" s="28"/>
+      <c r="F35" s="32"/>
+      <c r="G35" s="32"/>
+      <c r="H35" s="32"/>
+      <c r="I35" s="33"/>
     </row>
     <row r="36" spans="1:9" s="9" customFormat="1" ht="9" customHeight="1">
-      <c r="A36" s="47"/>
+      <c r="A36" s="51"/>
       <c r="B36" s="6"/>
       <c r="C36" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="D36" s="12" t="s">
+        <v>10</v>
+      </c>
+      <c r="D36" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="E36" s="22"/>
+      <c r="F36" s="32"/>
+      <c r="G36" s="32"/>
+      <c r="H36" s="32"/>
+      <c r="I36" s="33"/>
+    </row>
+    <row r="37" spans="1:9" s="9" customFormat="1" ht="9" customHeight="1">
+      <c r="A37" s="51"/>
+      <c r="B37" s="6"/>
+      <c r="C37" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="D37" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="E37" s="22"/>
+      <c r="F37" s="32"/>
+      <c r="G37" s="32"/>
+      <c r="H37" s="32"/>
+      <c r="I37" s="33"/>
+    </row>
+    <row r="38" spans="1:9" s="9" customFormat="1" ht="9" customHeight="1">
+      <c r="A38" s="51"/>
+      <c r="B38" s="6"/>
+      <c r="C38" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="D38" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="E38" s="22"/>
+      <c r="F38" s="32"/>
+      <c r="G38" s="32"/>
+      <c r="H38" s="32"/>
+      <c r="I38" s="33"/>
+    </row>
+    <row r="39" spans="1:9" s="9" customFormat="1" ht="9" customHeight="1">
+      <c r="A39" s="51"/>
+      <c r="B39" s="6"/>
+      <c r="C39" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="D39" s="12" t="s">
+        <v>40</v>
+      </c>
+      <c r="E39" s="22"/>
+      <c r="F39" s="32"/>
+      <c r="G39" s="32"/>
+      <c r="H39" s="32"/>
+      <c r="I39" s="33"/>
+    </row>
+    <row r="40" spans="1:9" s="9" customFormat="1" ht="9" customHeight="1">
+      <c r="A40" s="51"/>
+      <c r="B40" s="13"/>
+      <c r="C40" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="D40" s="8" t="s">
+        <v>41</v>
+      </c>
+      <c r="E40" s="22"/>
+      <c r="F40" s="32"/>
+      <c r="G40" s="32"/>
+      <c r="H40" s="32"/>
+      <c r="I40" s="33"/>
+    </row>
+    <row r="41" spans="1:9" s="9" customFormat="1" ht="9" customHeight="1">
+      <c r="A41" s="51"/>
+      <c r="B41" s="13"/>
+      <c r="C41" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="D41" s="8" t="s">
         <v>42</v>
       </c>
-      <c r="E36" s="22"/>
-      <c r="F36" s="27"/>
-      <c r="G36" s="27"/>
-      <c r="H36" s="27"/>
-      <c r="I36" s="28"/>
-    </row>
-    <row r="37" spans="1:9" s="9" customFormat="1" ht="9" customHeight="1">
-      <c r="A37" s="47"/>
-      <c r="B37" s="13"/>
-      <c r="C37" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="D37" s="8" t="s">
+      <c r="E41" s="25"/>
+      <c r="F41" s="32"/>
+      <c r="G41" s="32"/>
+      <c r="H41" s="32"/>
+      <c r="I41" s="33"/>
+    </row>
+    <row r="42" spans="1:9" s="9" customFormat="1" ht="9" customHeight="1">
+      <c r="A42" s="51"/>
+      <c r="B42" s="13"/>
+      <c r="C42" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="D42" s="8" t="s">
         <v>43</v>
       </c>
-      <c r="E37" s="22"/>
-      <c r="F37" s="27"/>
-      <c r="G37" s="27"/>
-      <c r="H37" s="27"/>
-      <c r="I37" s="28"/>
-    </row>
-    <row r="38" spans="1:9" s="9" customFormat="1" ht="9" customHeight="1">
-      <c r="A38" s="47"/>
-      <c r="B38" s="13"/>
-      <c r="C38" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="D38" s="8" t="s">
-        <v>44</v>
-      </c>
-      <c r="E38" s="25"/>
-      <c r="F38" s="27"/>
-      <c r="G38" s="27"/>
-      <c r="H38" s="27"/>
-      <c r="I38" s="28"/>
-    </row>
-    <row r="39" spans="1:9" s="9" customFormat="1" ht="9" customHeight="1">
-      <c r="A39" s="47"/>
-      <c r="B39" s="13"/>
-      <c r="C39" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="D39" s="8" t="s">
-        <v>45</v>
-      </c>
-      <c r="E39" s="25"/>
-      <c r="F39" s="27"/>
-      <c r="G39" s="27"/>
-      <c r="H39" s="27"/>
-      <c r="I39" s="28"/>
-    </row>
-    <row r="40" spans="1:9" s="9" customFormat="1" ht="9" customHeight="1">
-      <c r="A40" s="47"/>
-      <c r="B40" s="6"/>
-      <c r="C40" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="D40" s="8" t="s">
-        <v>46</v>
-      </c>
-      <c r="E40" s="22"/>
-      <c r="F40" s="27"/>
-      <c r="G40" s="27"/>
-      <c r="H40" s="27"/>
-      <c r="I40" s="28"/>
-    </row>
-    <row r="41" spans="1:9" s="9" customFormat="1" ht="9" customHeight="1">
-      <c r="A41" s="47"/>
-      <c r="B41" s="6"/>
-      <c r="C41" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="D41" s="8" t="s">
-        <v>47</v>
-      </c>
-      <c r="E41" s="22"/>
-      <c r="F41" s="27"/>
-      <c r="G41" s="27"/>
-      <c r="H41" s="27"/>
-      <c r="I41" s="28"/>
-    </row>
-    <row r="42" spans="1:9" s="9" customFormat="1" ht="9" customHeight="1">
-      <c r="A42" s="47"/>
-      <c r="B42" s="6"/>
-      <c r="C42" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="D42" s="8" t="s">
-        <v>48</v>
-      </c>
-      <c r="E42" s="22"/>
-      <c r="F42" s="27"/>
-      <c r="G42" s="27"/>
-      <c r="H42" s="27"/>
-      <c r="I42" s="28"/>
+      <c r="E42" s="25"/>
+      <c r="F42" s="32"/>
+      <c r="G42" s="32"/>
+      <c r="H42" s="32"/>
+      <c r="I42" s="33"/>
     </row>
     <row r="43" spans="1:9" s="9" customFormat="1" ht="9" customHeight="1">
-      <c r="A43" s="47"/>
+      <c r="A43" s="51"/>
       <c r="B43" s="6"/>
       <c r="C43" s="7" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D43" s="8" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="E43" s="22"/>
-      <c r="F43" s="27"/>
-      <c r="G43" s="27"/>
-      <c r="H43" s="27"/>
-      <c r="I43" s="28"/>
+      <c r="F43" s="32"/>
+      <c r="G43" s="32"/>
+      <c r="H43" s="32"/>
+      <c r="I43" s="33"/>
     </row>
     <row r="44" spans="1:9" s="9" customFormat="1" ht="9" customHeight="1">
-      <c r="A44" s="47"/>
+      <c r="A44" s="51"/>
       <c r="B44" s="6"/>
       <c r="C44" s="7" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D44" s="8" t="s">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="E44" s="22"/>
-      <c r="F44" s="27"/>
-      <c r="G44" s="27"/>
-      <c r="H44" s="27"/>
-      <c r="I44" s="28"/>
+      <c r="F44" s="32"/>
+      <c r="G44" s="32"/>
+      <c r="H44" s="32"/>
+      <c r="I44" s="33"/>
     </row>
     <row r="45" spans="1:9" s="9" customFormat="1" ht="9" customHeight="1">
-      <c r="A45" s="47"/>
+      <c r="A45" s="51"/>
       <c r="B45" s="6"/>
       <c r="C45" s="7" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D45" s="8" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
       <c r="E45" s="22"/>
-      <c r="F45" s="27"/>
-      <c r="G45" s="27"/>
-      <c r="H45" s="27"/>
-      <c r="I45" s="28"/>
+      <c r="F45" s="32"/>
+      <c r="G45" s="32"/>
+      <c r="H45" s="32"/>
+      <c r="I45" s="33"/>
     </row>
     <row r="46" spans="1:9" s="9" customFormat="1" ht="9" customHeight="1">
-      <c r="A46" s="47"/>
+      <c r="A46" s="51"/>
       <c r="B46" s="6"/>
       <c r="C46" s="7" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D46" s="8" t="s">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="E46" s="22"/>
-      <c r="F46" s="27"/>
-      <c r="G46" s="27"/>
-      <c r="H46" s="27"/>
-      <c r="I46" s="28"/>
+      <c r="F46" s="32"/>
+      <c r="G46" s="32"/>
+      <c r="H46" s="32"/>
+      <c r="I46" s="33"/>
     </row>
     <row r="47" spans="1:9" s="9" customFormat="1" ht="9" customHeight="1">
-      <c r="A47" s="47"/>
+      <c r="A47" s="51"/>
       <c r="B47" s="6"/>
       <c r="C47" s="7" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D47" s="8" t="s">
-        <v>53</v>
+        <v>48</v>
       </c>
       <c r="E47" s="22"/>
-      <c r="F47" s="27"/>
-      <c r="G47" s="27"/>
-      <c r="H47" s="27"/>
-      <c r="I47" s="28"/>
+      <c r="F47" s="32"/>
+      <c r="G47" s="32"/>
+      <c r="H47" s="32"/>
+      <c r="I47" s="33"/>
     </row>
     <row r="48" spans="1:9" s="9" customFormat="1" ht="9" customHeight="1">
-      <c r="A48" s="47"/>
+      <c r="A48" s="51"/>
       <c r="B48" s="6"/>
       <c r="C48" s="7" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D48" s="8" t="s">
-        <v>54</v>
+        <v>49</v>
       </c>
       <c r="E48" s="22"/>
-      <c r="F48" s="27"/>
-      <c r="G48" s="27"/>
-      <c r="H48" s="27"/>
-      <c r="I48" s="28"/>
+      <c r="F48" s="32"/>
+      <c r="G48" s="32"/>
+      <c r="H48" s="32"/>
+      <c r="I48" s="33"/>
     </row>
     <row r="49" spans="1:9" s="9" customFormat="1" ht="9" customHeight="1">
-      <c r="A49" s="47"/>
+      <c r="A49" s="51"/>
       <c r="B49" s="6"/>
       <c r="C49" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="D49" s="14" t="s">
+        <v>10</v>
+      </c>
+      <c r="D49" s="8" t="s">
+        <v>50</v>
+      </c>
+      <c r="E49" s="22"/>
+      <c r="F49" s="32"/>
+      <c r="G49" s="32"/>
+      <c r="H49" s="32"/>
+      <c r="I49" s="33"/>
+    </row>
+    <row r="50" spans="1:9" s="9" customFormat="1" ht="9" customHeight="1">
+      <c r="A50" s="51"/>
+      <c r="B50" s="6"/>
+      <c r="C50" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="D50" s="8" t="s">
+        <v>51</v>
+      </c>
+      <c r="E50" s="22"/>
+      <c r="F50" s="32"/>
+      <c r="G50" s="32"/>
+      <c r="H50" s="32"/>
+      <c r="I50" s="33"/>
+    </row>
+    <row r="51" spans="1:9" s="9" customFormat="1" ht="9" customHeight="1">
+      <c r="A51" s="51"/>
+      <c r="B51" s="6"/>
+      <c r="C51" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="D51" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="E51" s="22"/>
+      <c r="F51" s="32"/>
+      <c r="G51" s="32"/>
+      <c r="H51" s="32"/>
+      <c r="I51" s="33"/>
+    </row>
+    <row r="52" spans="1:9" s="9" customFormat="1" ht="9" customHeight="1">
+      <c r="A52" s="51"/>
+      <c r="B52" s="6"/>
+      <c r="C52" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="D52" s="14" t="s">
+        <v>53</v>
+      </c>
+      <c r="E52" s="22"/>
+      <c r="F52" s="32"/>
+      <c r="G52" s="32"/>
+      <c r="H52" s="32"/>
+      <c r="I52" s="33"/>
+    </row>
+    <row r="53" spans="1:9" s="9" customFormat="1" ht="9" customHeight="1">
+      <c r="A53" s="51"/>
+      <c r="B53" s="6"/>
+      <c r="C53" s="15" t="s">
+        <v>10</v>
+      </c>
+      <c r="D53" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="E53" s="22"/>
+      <c r="F53" s="32"/>
+      <c r="G53" s="32"/>
+      <c r="H53" s="32"/>
+      <c r="I53" s="33"/>
+    </row>
+    <row r="54" spans="1:9" s="9" customFormat="1" ht="9" customHeight="1">
+      <c r="A54" s="51"/>
+      <c r="B54" s="6"/>
+      <c r="C54" s="7"/>
+      <c r="D54" s="14"/>
+      <c r="E54" s="22"/>
+      <c r="F54" s="32"/>
+      <c r="G54" s="32"/>
+      <c r="H54" s="32"/>
+      <c r="I54" s="33"/>
+    </row>
+    <row r="55" spans="1:9" s="9" customFormat="1" ht="9" customHeight="1">
+      <c r="A55" s="51"/>
+      <c r="B55" s="6"/>
+      <c r="C55" s="17"/>
+      <c r="D55" s="18"/>
+      <c r="E55" s="22"/>
+      <c r="F55" s="32"/>
+      <c r="G55" s="32"/>
+      <c r="H55" s="32"/>
+      <c r="I55" s="33"/>
+    </row>
+    <row r="56" spans="1:9" s="9" customFormat="1" ht="9" customHeight="1">
+      <c r="A56" s="54" t="s">
         <v>55</v>
       </c>
-      <c r="E49" s="22"/>
-      <c r="F49" s="27"/>
-      <c r="G49" s="27"/>
-      <c r="H49" s="27"/>
-      <c r="I49" s="28"/>
-    </row>
-    <row r="50" spans="1:9" s="9" customFormat="1" ht="9" customHeight="1">
-      <c r="A50" s="47"/>
-      <c r="B50" s="6"/>
-      <c r="C50" s="15" t="s">
-        <v>12</v>
-      </c>
-      <c r="D50" s="16" t="s">
+      <c r="B56" s="6"/>
+      <c r="C56" s="55" t="s">
         <v>56</v>
       </c>
-      <c r="E50" s="22"/>
-      <c r="F50" s="27"/>
-      <c r="G50" s="27"/>
-      <c r="H50" s="27"/>
-      <c r="I50" s="28"/>
-    </row>
-    <row r="51" spans="1:9" s="9" customFormat="1" ht="9" customHeight="1">
-      <c r="A51" s="47"/>
-      <c r="B51" s="6"/>
-      <c r="C51" s="7"/>
-      <c r="D51" s="14"/>
-      <c r="E51" s="22"/>
-      <c r="F51" s="27"/>
-      <c r="G51" s="27"/>
-      <c r="H51" s="27"/>
-      <c r="I51" s="28"/>
-    </row>
-    <row r="52" spans="1:9" s="9" customFormat="1" ht="9" customHeight="1">
-      <c r="A52" s="47"/>
-      <c r="B52" s="6"/>
-      <c r="C52" s="17"/>
-      <c r="D52" s="18"/>
-      <c r="E52" s="22"/>
-      <c r="F52" s="27"/>
-      <c r="G52" s="27"/>
-      <c r="H52" s="27"/>
-      <c r="I52" s="28"/>
-    </row>
-    <row r="53" spans="1:9" s="9" customFormat="1" ht="9" customHeight="1">
-      <c r="A53" s="50" t="s">
+      <c r="D56" s="55"/>
+      <c r="E56" s="22"/>
+      <c r="F56" s="32"/>
+      <c r="G56" s="32"/>
+      <c r="H56" s="32"/>
+      <c r="I56" s="33"/>
+    </row>
+    <row r="57" spans="1:9" s="9" customFormat="1" ht="9" customHeight="1">
+      <c r="A57" s="54"/>
+      <c r="B57" s="6"/>
+      <c r="C57" s="55" t="s">
         <v>57</v>
       </c>
-      <c r="B53" s="6"/>
-      <c r="C53" s="51" t="s">
+      <c r="D57" s="55"/>
+      <c r="E57" s="22"/>
+      <c r="F57" s="32"/>
+      <c r="G57" s="32"/>
+      <c r="H57" s="32"/>
+      <c r="I57" s="33"/>
+    </row>
+    <row r="58" spans="1:9" s="9" customFormat="1" ht="9" customHeight="1">
+      <c r="A58" s="54"/>
+      <c r="B58" s="6"/>
+      <c r="C58" s="55" t="s">
         <v>58</v>
       </c>
-      <c r="D53" s="51"/>
-      <c r="E53" s="22"/>
-      <c r="F53" s="27"/>
-      <c r="G53" s="27"/>
-      <c r="H53" s="27"/>
-      <c r="I53" s="28"/>
-    </row>
-    <row r="54" spans="1:9" s="9" customFormat="1" ht="9" customHeight="1">
-      <c r="A54" s="50"/>
-      <c r="B54" s="6"/>
-      <c r="C54" s="51" t="s">
+      <c r="D58" s="55"/>
+      <c r="E58" s="22"/>
+      <c r="F58" s="32"/>
+      <c r="G58" s="32"/>
+      <c r="H58" s="32"/>
+      <c r="I58" s="33"/>
+    </row>
+    <row r="59" spans="1:9" s="9" customFormat="1" ht="9" customHeight="1">
+      <c r="A59" s="54"/>
+      <c r="B59" s="13"/>
+      <c r="C59" s="55" t="s">
         <v>59</v>
       </c>
-      <c r="D54" s="51"/>
-      <c r="E54" s="22"/>
-      <c r="F54" s="27"/>
-      <c r="G54" s="27"/>
-      <c r="H54" s="27"/>
-      <c r="I54" s="28"/>
-    </row>
-    <row r="55" spans="1:9" s="9" customFormat="1" ht="9" customHeight="1">
-      <c r="A55" s="50"/>
-      <c r="B55" s="6"/>
-      <c r="C55" s="51" t="s">
-        <v>60</v>
-      </c>
-      <c r="D55" s="51"/>
-      <c r="E55" s="22"/>
-      <c r="F55" s="27"/>
-      <c r="G55" s="27"/>
-      <c r="H55" s="27"/>
-      <c r="I55" s="28"/>
-    </row>
-    <row r="56" spans="1:9" s="9" customFormat="1" ht="9" customHeight="1">
-      <c r="A56" s="50"/>
-      <c r="B56" s="13"/>
-      <c r="C56" s="51" t="s">
-        <v>61</v>
-      </c>
-      <c r="D56" s="51"/>
-      <c r="E56" s="25"/>
-      <c r="F56" s="27"/>
-      <c r="G56" s="27"/>
-      <c r="H56" s="27"/>
-      <c r="I56" s="28"/>
-    </row>
-    <row r="57" spans="1:9" ht="9" customHeight="1">
-      <c r="A57" s="58"/>
-      <c r="B57" s="19"/>
-      <c r="C57" s="60"/>
-      <c r="D57" s="61"/>
-      <c r="E57" s="24"/>
-      <c r="F57" s="62"/>
-      <c r="G57" s="62"/>
-      <c r="H57" s="62"/>
-      <c r="I57" s="63"/>
-    </row>
-    <row r="58" spans="1:9" ht="9" customHeight="1">
-      <c r="A58" s="58"/>
-      <c r="B58" s="19"/>
-      <c r="C58" s="60"/>
-      <c r="D58" s="61"/>
-      <c r="E58" s="24"/>
-      <c r="F58" s="64"/>
-      <c r="G58" s="64"/>
-      <c r="H58" s="64"/>
-      <c r="I58" s="65"/>
-    </row>
-    <row r="59" spans="1:9" ht="9" customHeight="1">
-      <c r="A59" s="58"/>
-      <c r="B59" s="19"/>
-      <c r="C59" s="60"/>
-      <c r="D59" s="61"/>
-      <c r="E59" s="23"/>
-      <c r="F59" s="52"/>
-      <c r="G59" s="52"/>
-      <c r="H59" s="52"/>
-      <c r="I59" s="53"/>
+      <c r="D59" s="55"/>
+      <c r="E59" s="25"/>
+      <c r="F59" s="32"/>
+      <c r="G59" s="32"/>
+      <c r="H59" s="32"/>
+      <c r="I59" s="33"/>
     </row>
     <row r="60" spans="1:9" ht="9" customHeight="1">
-      <c r="A60" s="58"/>
+      <c r="A60" s="71"/>
       <c r="B60" s="19"/>
-      <c r="C60" s="60"/>
-      <c r="D60" s="61"/>
-      <c r="E60" s="23"/>
-      <c r="F60" s="52"/>
-      <c r="G60" s="52"/>
-      <c r="H60" s="52"/>
-      <c r="I60" s="53"/>
+      <c r="C60" s="73"/>
+      <c r="D60" s="74"/>
+      <c r="E60" s="24"/>
+      <c r="F60" s="75"/>
+      <c r="G60" s="75"/>
+      <c r="H60" s="75"/>
+      <c r="I60" s="76"/>
     </row>
     <row r="61" spans="1:9" ht="9" customHeight="1">
-      <c r="A61" s="59"/>
+      <c r="A61" s="71"/>
       <c r="B61" s="19"/>
-      <c r="C61" s="60"/>
-      <c r="D61" s="61"/>
-      <c r="E61" s="23"/>
-      <c r="F61" s="52"/>
-      <c r="G61" s="52"/>
-      <c r="H61" s="52"/>
-      <c r="I61" s="53"/>
+      <c r="C61" s="73"/>
+      <c r="D61" s="74"/>
+      <c r="E61" s="24"/>
+      <c r="F61" s="77"/>
+      <c r="G61" s="77"/>
+      <c r="H61" s="77"/>
+      <c r="I61" s="78"/>
     </row>
     <row r="62" spans="1:9" ht="9" customHeight="1">
-      <c r="A62" s="70" t="s">
-        <v>62</v>
-      </c>
-      <c r="B62" s="71"/>
-      <c r="C62" s="71"/>
-      <c r="D62" s="72"/>
-      <c r="E62" s="54" t="s">
-        <v>63</v>
-      </c>
-      <c r="F62" s="54"/>
-      <c r="G62" s="54"/>
-      <c r="H62" s="54"/>
-      <c r="I62" s="55"/>
+      <c r="A62" s="71"/>
+      <c r="B62" s="19"/>
+      <c r="C62" s="73"/>
+      <c r="D62" s="74"/>
+      <c r="E62" s="23"/>
+      <c r="F62" s="56"/>
+      <c r="G62" s="56"/>
+      <c r="H62" s="56"/>
+      <c r="I62" s="57"/>
     </row>
     <row r="63" spans="1:9" ht="9" customHeight="1">
-      <c r="A63" s="73"/>
-      <c r="B63" s="74"/>
-      <c r="C63" s="74"/>
-      <c r="D63" s="75"/>
-      <c r="E63" s="43" t="s">
-        <v>64</v>
-      </c>
-      <c r="F63" s="43"/>
-      <c r="G63" s="43"/>
-      <c r="H63" s="43"/>
-      <c r="I63" s="4" t="s">
-        <v>65</v>
-      </c>
+      <c r="A63" s="71"/>
+      <c r="B63" s="19"/>
+      <c r="C63" s="73"/>
+      <c r="D63" s="74"/>
+      <c r="E63" s="23"/>
+      <c r="F63" s="56"/>
+      <c r="G63" s="56"/>
+      <c r="H63" s="56"/>
+      <c r="I63" s="57"/>
     </row>
     <row r="64" spans="1:9" ht="9" customHeight="1">
-      <c r="A64" s="73"/>
-      <c r="B64" s="74"/>
-      <c r="C64" s="74"/>
-      <c r="D64" s="75"/>
-      <c r="E64" s="56"/>
+      <c r="A64" s="72"/>
+      <c r="B64" s="19"/>
+      <c r="C64" s="73"/>
+      <c r="D64" s="74"/>
+      <c r="E64" s="23"/>
       <c r="F64" s="56"/>
       <c r="G64" s="56"/>
       <c r="H64" s="56"/>
-      <c r="I64" s="20"/>
+      <c r="I64" s="57"/>
     </row>
     <row r="65" spans="1:9" ht="9" customHeight="1">
-      <c r="A65" s="73"/>
-      <c r="B65" s="74"/>
-      <c r="C65" s="74"/>
-      <c r="D65" s="75"/>
-      <c r="E65" s="56"/>
-      <c r="F65" s="56"/>
-      <c r="G65" s="56"/>
-      <c r="H65" s="56"/>
-      <c r="I65" s="20"/>
+      <c r="A65" s="58" t="s">
+        <v>60</v>
+      </c>
+      <c r="B65" s="59"/>
+      <c r="C65" s="59"/>
+      <c r="D65" s="60"/>
+      <c r="E65" s="67" t="s">
+        <v>61</v>
+      </c>
+      <c r="F65" s="67"/>
+      <c r="G65" s="67"/>
+      <c r="H65" s="67"/>
+      <c r="I65" s="68"/>
     </row>
     <row r="66" spans="1:9" ht="9" customHeight="1">
-      <c r="A66" s="73"/>
-      <c r="B66" s="74"/>
-      <c r="C66" s="74"/>
-      <c r="D66" s="75"/>
-      <c r="E66" s="56"/>
-      <c r="F66" s="56"/>
-      <c r="G66" s="56"/>
-      <c r="H66" s="56"/>
-      <c r="I66" s="20"/>
+      <c r="A66" s="61"/>
+      <c r="B66" s="62"/>
+      <c r="C66" s="62"/>
+      <c r="D66" s="63"/>
+      <c r="E66" s="48" t="s">
+        <v>62</v>
+      </c>
+      <c r="F66" s="48"/>
+      <c r="G66" s="48"/>
+      <c r="H66" s="48"/>
+      <c r="I66" s="4" t="s">
+        <v>63</v>
+      </c>
     </row>
     <row r="67" spans="1:9" ht="9" customHeight="1">
-      <c r="A67" s="73"/>
-      <c r="B67" s="74"/>
-      <c r="C67" s="74"/>
-      <c r="D67" s="75"/>
-      <c r="E67" s="56"/>
-      <c r="F67" s="56"/>
-      <c r="G67" s="56"/>
-      <c r="H67" s="56"/>
+      <c r="A67" s="61"/>
+      <c r="B67" s="62"/>
+      <c r="C67" s="62"/>
+      <c r="D67" s="63"/>
+      <c r="E67" s="69"/>
+      <c r="F67" s="69"/>
+      <c r="G67" s="69"/>
+      <c r="H67" s="69"/>
       <c r="I67" s="20"/>
     </row>
     <row r="68" spans="1:9" ht="9" customHeight="1">
-      <c r="A68" s="73"/>
-      <c r="B68" s="74"/>
-      <c r="C68" s="74"/>
-      <c r="D68" s="75"/>
-      <c r="E68" s="56"/>
-      <c r="F68" s="56"/>
-      <c r="G68" s="56"/>
-      <c r="H68" s="56"/>
+      <c r="A68" s="61"/>
+      <c r="B68" s="62"/>
+      <c r="C68" s="62"/>
+      <c r="D68" s="63"/>
+      <c r="E68" s="69"/>
+      <c r="F68" s="69"/>
+      <c r="G68" s="69"/>
+      <c r="H68" s="69"/>
       <c r="I68" s="20"/>
     </row>
     <row r="69" spans="1:9" ht="9" customHeight="1">
-      <c r="A69" s="73"/>
-      <c r="B69" s="74"/>
-      <c r="C69" s="74"/>
-      <c r="D69" s="75"/>
-      <c r="E69" s="57" t="s">
+      <c r="A69" s="61"/>
+      <c r="B69" s="62"/>
+      <c r="C69" s="62"/>
+      <c r="D69" s="63"/>
+      <c r="E69" s="69"/>
+      <c r="F69" s="69"/>
+      <c r="G69" s="69"/>
+      <c r="H69" s="69"/>
+      <c r="I69" s="20"/>
+    </row>
+    <row r="70" spans="1:9" ht="9" customHeight="1">
+      <c r="A70" s="61"/>
+      <c r="B70" s="62"/>
+      <c r="C70" s="62"/>
+      <c r="D70" s="63"/>
+      <c r="E70" s="69"/>
+      <c r="F70" s="69"/>
+      <c r="G70" s="69"/>
+      <c r="H70" s="69"/>
+      <c r="I70" s="20"/>
+    </row>
+    <row r="71" spans="1:9" ht="9" customHeight="1">
+      <c r="A71" s="61"/>
+      <c r="B71" s="62"/>
+      <c r="C71" s="62"/>
+      <c r="D71" s="63"/>
+      <c r="E71" s="69"/>
+      <c r="F71" s="69"/>
+      <c r="G71" s="69"/>
+      <c r="H71" s="69"/>
+      <c r="I71" s="20"/>
+    </row>
+    <row r="72" spans="1:9" ht="9" customHeight="1">
+      <c r="A72" s="61"/>
+      <c r="B72" s="62"/>
+      <c r="C72" s="62"/>
+      <c r="D72" s="63"/>
+      <c r="E72" s="70" t="s">
+        <v>64</v>
+      </c>
+      <c r="F72" s="70"/>
+      <c r="G72" s="70"/>
+      <c r="H72" s="32"/>
+      <c r="I72" s="33"/>
+    </row>
+    <row r="73" spans="1:9" ht="9" customHeight="1">
+      <c r="A73" s="61"/>
+      <c r="B73" s="62"/>
+      <c r="C73" s="62"/>
+      <c r="D73" s="63"/>
+      <c r="E73" s="70" t="s">
+        <v>65</v>
+      </c>
+      <c r="F73" s="70"/>
+      <c r="G73" s="70"/>
+      <c r="H73" s="32"/>
+      <c r="I73" s="33"/>
+    </row>
+    <row r="74" spans="1:9" ht="9" customHeight="1">
+      <c r="A74" s="61"/>
+      <c r="B74" s="62"/>
+      <c r="C74" s="62"/>
+      <c r="D74" s="63"/>
+      <c r="E74" s="70" t="s">
         <v>66</v>
       </c>
-      <c r="F69" s="57"/>
-      <c r="G69" s="57"/>
-      <c r="H69" s="27"/>
-      <c r="I69" s="28"/>
-    </row>
-    <row r="70" spans="1:9" ht="9" customHeight="1">
-      <c r="A70" s="73"/>
-      <c r="B70" s="74"/>
-      <c r="C70" s="74"/>
-      <c r="D70" s="75"/>
-      <c r="E70" s="57" t="s">
+      <c r="F74" s="70"/>
+      <c r="G74" s="70"/>
+      <c r="H74" s="32"/>
+      <c r="I74" s="33"/>
+    </row>
+    <row r="75" spans="1:9" ht="9" customHeight="1">
+      <c r="A75" s="61"/>
+      <c r="B75" s="62"/>
+      <c r="C75" s="62"/>
+      <c r="D75" s="63"/>
+      <c r="E75" s="70" t="s">
         <v>67</v>
       </c>
-      <c r="F70" s="57"/>
-      <c r="G70" s="57"/>
-      <c r="H70" s="27"/>
-      <c r="I70" s="28"/>
-    </row>
-    <row r="71" spans="1:9" ht="9" customHeight="1">
-      <c r="A71" s="73"/>
-      <c r="B71" s="74"/>
-      <c r="C71" s="74"/>
-      <c r="D71" s="75"/>
-      <c r="E71" s="57" t="s">
+      <c r="F75" s="70"/>
+      <c r="G75" s="70"/>
+      <c r="H75" s="32"/>
+      <c r="I75" s="33"/>
+    </row>
+    <row r="76" spans="1:9" ht="9" customHeight="1">
+      <c r="A76" s="61"/>
+      <c r="B76" s="62"/>
+      <c r="C76" s="62"/>
+      <c r="D76" s="63"/>
+      <c r="E76" s="70" t="s">
         <v>68</v>
       </c>
-      <c r="F71" s="57"/>
-      <c r="G71" s="57"/>
-      <c r="H71" s="27"/>
-      <c r="I71" s="28"/>
-    </row>
-    <row r="72" spans="1:9" ht="9" customHeight="1">
-      <c r="A72" s="73"/>
-      <c r="B72" s="74"/>
-      <c r="C72" s="74"/>
-      <c r="D72" s="75"/>
-      <c r="E72" s="57" t="s">
+      <c r="F76" s="70"/>
+      <c r="G76" s="70"/>
+      <c r="H76" s="32"/>
+      <c r="I76" s="33"/>
+    </row>
+    <row r="77" spans="1:9" ht="9" customHeight="1" thickBot="1">
+      <c r="A77" s="64"/>
+      <c r="B77" s="65"/>
+      <c r="C77" s="65"/>
+      <c r="D77" s="66"/>
+      <c r="E77" s="82" t="s">
         <v>69</v>
       </c>
-      <c r="F72" s="57"/>
-      <c r="G72" s="57"/>
-      <c r="H72" s="27"/>
-      <c r="I72" s="28"/>
-    </row>
-    <row r="73" spans="1:9" ht="9" customHeight="1">
-      <c r="A73" s="73"/>
-      <c r="B73" s="74"/>
-      <c r="C73" s="74"/>
-      <c r="D73" s="75"/>
-      <c r="E73" s="57" t="s">
+      <c r="F77" s="82"/>
+      <c r="G77" s="82"/>
+      <c r="H77" s="80"/>
+      <c r="I77" s="81"/>
+    </row>
+    <row r="78" spans="1:9" ht="9" customHeight="1" thickTop="1">
+      <c r="G78" s="79" t="s">
         <v>70</v>
       </c>
-      <c r="F73" s="57"/>
-      <c r="G73" s="57"/>
-      <c r="H73" s="27"/>
-      <c r="I73" s="28"/>
-    </row>
-    <row r="74" spans="1:9" ht="9" customHeight="1" thickBot="1">
-      <c r="A74" s="76"/>
-      <c r="B74" s="77"/>
-      <c r="C74" s="77"/>
-      <c r="D74" s="78"/>
-      <c r="E74" s="69" t="s">
-        <v>71</v>
-      </c>
-      <c r="F74" s="69"/>
-      <c r="G74" s="69"/>
-      <c r="H74" s="67"/>
-      <c r="I74" s="68"/>
-    </row>
-    <row r="75" spans="1:9" ht="9" customHeight="1" thickTop="1">
-      <c r="G75" s="66" t="s">
-        <v>72</v>
-      </c>
-      <c r="H75" s="66"/>
-      <c r="I75" s="66"/>
-    </row>
-    <row r="76" spans="1:9" ht="9" customHeight="1">
-      <c r="A76"/>
-      <c r="B76"/>
-      <c r="C76"/>
-      <c r="D76"/>
-      <c r="E76"/>
-      <c r="F76"/>
-      <c r="G76"/>
-      <c r="H76"/>
-      <c r="I76"/>
-    </row>
-    <row r="77" spans="1:9">
-      <c r="A77"/>
-      <c r="B77"/>
-      <c r="C77"/>
-      <c r="D77"/>
-      <c r="E77"/>
-      <c r="F77"/>
-      <c r="G77"/>
-      <c r="H77"/>
-      <c r="I77"/>
-    </row>
-    <row r="78" spans="1:9">
-      <c r="A78"/>
-      <c r="B78"/>
-      <c r="C78"/>
-      <c r="D78"/>
-      <c r="E78"/>
-      <c r="F78"/>
-      <c r="G78"/>
-      <c r="H78"/>
-      <c r="I78"/>
-    </row>
-    <row r="79" spans="1:9">
+      <c r="H78" s="79"/>
+      <c r="I78" s="79"/>
+    </row>
+    <row r="79" spans="1:9" ht="9" customHeight="1">
       <c r="A79"/>
       <c r="B79"/>
       <c r="C79"/>
@@ -2400,113 +2450,125 @@
     <row r="81" customFormat="1"/>
     <row r="82" customFormat="1"/>
     <row r="83" customFormat="1"/>
+    <row r="84" customFormat="1"/>
+    <row r="85" customFormat="1"/>
+    <row r="86" customFormat="1"/>
   </sheetData>
-  <mergeCells count="105">
-    <mergeCell ref="G75:I75"/>
-    <mergeCell ref="H69:I70"/>
-    <mergeCell ref="E70:G70"/>
-    <mergeCell ref="E71:G71"/>
-    <mergeCell ref="H71:I72"/>
-    <mergeCell ref="E72:G72"/>
+  <mergeCells count="114">
+    <mergeCell ref="G78:I78"/>
+    <mergeCell ref="H72:I73"/>
     <mergeCell ref="E73:G73"/>
-    <mergeCell ref="H73:I74"/>
     <mergeCell ref="E74:G74"/>
-    <mergeCell ref="F61:I61"/>
-    <mergeCell ref="A62:D74"/>
-    <mergeCell ref="E62:I62"/>
-    <mergeCell ref="E63:H63"/>
-    <mergeCell ref="E64:H64"/>
-    <mergeCell ref="E65:H65"/>
+    <mergeCell ref="H74:I75"/>
+    <mergeCell ref="E75:G75"/>
+    <mergeCell ref="E76:G76"/>
+    <mergeCell ref="H76:I77"/>
+    <mergeCell ref="E77:G77"/>
+    <mergeCell ref="F64:I64"/>
+    <mergeCell ref="A65:D77"/>
+    <mergeCell ref="E65:I65"/>
     <mergeCell ref="E66:H66"/>
     <mergeCell ref="E67:H67"/>
     <mergeCell ref="E68:H68"/>
-    <mergeCell ref="E69:G69"/>
-    <mergeCell ref="A57:A61"/>
+    <mergeCell ref="E69:H69"/>
+    <mergeCell ref="E70:H70"/>
+    <mergeCell ref="E71:H71"/>
+    <mergeCell ref="E72:G72"/>
+    <mergeCell ref="A60:A64"/>
+    <mergeCell ref="C60:D60"/>
+    <mergeCell ref="F60:I60"/>
+    <mergeCell ref="C61:D61"/>
+    <mergeCell ref="F61:I61"/>
+    <mergeCell ref="C62:D62"/>
+    <mergeCell ref="F62:I62"/>
+    <mergeCell ref="C63:D63"/>
+    <mergeCell ref="F63:I63"/>
+    <mergeCell ref="C64:D64"/>
+    <mergeCell ref="F55:I55"/>
+    <mergeCell ref="A56:A59"/>
+    <mergeCell ref="C56:D56"/>
+    <mergeCell ref="F56:I56"/>
     <mergeCell ref="C57:D57"/>
     <mergeCell ref="F57:I57"/>
     <mergeCell ref="C58:D58"/>
     <mergeCell ref="F58:I58"/>
     <mergeCell ref="C59:D59"/>
     <mergeCell ref="F59:I59"/>
-    <mergeCell ref="C60:D60"/>
-    <mergeCell ref="F60:I60"/>
-    <mergeCell ref="C61:D61"/>
+    <mergeCell ref="A33:A55"/>
+    <mergeCell ref="F49:I49"/>
+    <mergeCell ref="F50:I50"/>
+    <mergeCell ref="F51:I51"/>
     <mergeCell ref="F52:I52"/>
-    <mergeCell ref="A53:A56"/>
-    <mergeCell ref="C53:D53"/>
     <mergeCell ref="F53:I53"/>
-    <mergeCell ref="C54:D54"/>
     <mergeCell ref="F54:I54"/>
-    <mergeCell ref="C55:D55"/>
-    <mergeCell ref="F55:I55"/>
-    <mergeCell ref="C56:D56"/>
-    <mergeCell ref="F56:I56"/>
-    <mergeCell ref="A30:A52"/>
+    <mergeCell ref="F43:I43"/>
+    <mergeCell ref="F44:I44"/>
+    <mergeCell ref="F45:I45"/>
     <mergeCell ref="F46:I46"/>
     <mergeCell ref="F47:I47"/>
     <mergeCell ref="F48:I48"/>
-    <mergeCell ref="F49:I49"/>
-    <mergeCell ref="F50:I50"/>
-    <mergeCell ref="F51:I51"/>
+    <mergeCell ref="F37:I37"/>
+    <mergeCell ref="F38:I38"/>
+    <mergeCell ref="F39:I39"/>
     <mergeCell ref="F40:I40"/>
     <mergeCell ref="F41:I41"/>
     <mergeCell ref="F42:I42"/>
-    <mergeCell ref="F43:I43"/>
-    <mergeCell ref="F44:I44"/>
-    <mergeCell ref="F45:I45"/>
+    <mergeCell ref="F29:I29"/>
+    <mergeCell ref="L29:M29"/>
+    <mergeCell ref="F30:I30"/>
+    <mergeCell ref="F31:I31"/>
+    <mergeCell ref="F32:I32"/>
+    <mergeCell ref="F33:I33"/>
     <mergeCell ref="F34:I34"/>
     <mergeCell ref="F35:I35"/>
     <mergeCell ref="F36:I36"/>
-    <mergeCell ref="F37:I37"/>
-    <mergeCell ref="F38:I38"/>
-    <mergeCell ref="F39:I39"/>
+    <mergeCell ref="F25:I25"/>
+    <mergeCell ref="L25:M25"/>
     <mergeCell ref="F26:I26"/>
     <mergeCell ref="L26:M26"/>
     <mergeCell ref="F27:I27"/>
     <mergeCell ref="F28:I28"/>
-    <mergeCell ref="F29:I29"/>
-    <mergeCell ref="F30:I30"/>
-    <mergeCell ref="F31:I31"/>
-    <mergeCell ref="F32:I32"/>
-    <mergeCell ref="F33:I33"/>
+    <mergeCell ref="A19:A32"/>
+    <mergeCell ref="F19:I19"/>
+    <mergeCell ref="L19:M19"/>
+    <mergeCell ref="F20:I20"/>
+    <mergeCell ref="L20:M20"/>
+    <mergeCell ref="F21:I21"/>
+    <mergeCell ref="L21:M21"/>
     <mergeCell ref="F22:I22"/>
-    <mergeCell ref="L22:M22"/>
     <mergeCell ref="F23:I23"/>
-    <mergeCell ref="L23:M23"/>
     <mergeCell ref="F24:I24"/>
-    <mergeCell ref="F25:I25"/>
-    <mergeCell ref="A16:A29"/>
-    <mergeCell ref="F16:I16"/>
-    <mergeCell ref="L16:M16"/>
-    <mergeCell ref="F17:I17"/>
-    <mergeCell ref="L17:M17"/>
-    <mergeCell ref="F18:I18"/>
-    <mergeCell ref="L18:M18"/>
-    <mergeCell ref="F19:I19"/>
-    <mergeCell ref="F20:I20"/>
-    <mergeCell ref="F21:I21"/>
-    <mergeCell ref="A6:A15"/>
-    <mergeCell ref="F6:I6"/>
-    <mergeCell ref="F7:I7"/>
-    <mergeCell ref="F8:I8"/>
+    <mergeCell ref="A9:A18"/>
     <mergeCell ref="F9:I9"/>
+    <mergeCell ref="F10:I10"/>
+    <mergeCell ref="F11:I11"/>
+    <mergeCell ref="F12:I12"/>
     <mergeCell ref="A1:C2"/>
     <mergeCell ref="D1:I1"/>
     <mergeCell ref="D2:I2"/>
     <mergeCell ref="E3:F3"/>
     <mergeCell ref="G3:I3"/>
-    <mergeCell ref="F10:I10"/>
-    <mergeCell ref="F11:I11"/>
-    <mergeCell ref="F12:I12"/>
     <mergeCell ref="F13:I13"/>
     <mergeCell ref="F14:I14"/>
     <mergeCell ref="F15:I15"/>
+    <mergeCell ref="F16:I16"/>
+    <mergeCell ref="F17:I17"/>
+    <mergeCell ref="F18:I18"/>
+    <mergeCell ref="E6:F6"/>
+    <mergeCell ref="G7:I7"/>
+    <mergeCell ref="B8:D8"/>
+    <mergeCell ref="F8:I8"/>
+    <mergeCell ref="C4:D4"/>
+    <mergeCell ref="C5:D5"/>
+    <mergeCell ref="C7:D7"/>
+    <mergeCell ref="E7:F7"/>
     <mergeCell ref="E4:F4"/>
+    <mergeCell ref="E5:F5"/>
     <mergeCell ref="G4:I4"/>
-    <mergeCell ref="B5:D5"/>
-    <mergeCell ref="F5:I5"/>
-    <mergeCell ref="B3:D3"/>
-    <mergeCell ref="B4:D4"/>
+    <mergeCell ref="G5:I5"/>
+    <mergeCell ref="G6:I6"/>
+    <mergeCell ref="C3:D3"/>
+    <mergeCell ref="C6:D6"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0" right="0" top="0.43263888888888902" bottom="0" header="0" footer="0"/>

</xml_diff>